<commit_message>
Documents-requested email, dependency upgrades, CI + Dependabot, web and app tests
- B2: "More documents needed" email to the company when staff request KYC
  documents (email event 5), staff note included.
- firebase-admin 13 -> 14 (push client on the modular API; Node >= 22).
  0 high/critical advisories in backend and web.
- CI workflow (backend with Mongo/Redis, web, app) with a high-severity audit
  gate; Dependabot for backend, web, app (security only) and Actions.
- Backend tests no longer depend on a developer .env (CORS/logo pinned in
  setup); test timeout 60 s.
- Web tests 42 -> 79 (server-parity checks for permissions, KYC documents and
  document names; signup, sign-in, permission gating, D6, chat files,
  quotation words). App: vitest + 16 logic tests (https-only release builds,
  log redaction, money, masking, validation).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/security-tracker.xlsx
+++ b/docs/security-tracker.xlsx
@@ -1706,18 +1706,22 @@
       </c>
       <c r="G18" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H18" s="32" t="inlineStr">
         <is>
-          <t>npm audit run 2026-09-25. Backend: 3 HIGH fixed the same day (multer 2.4.0, nodemailer 9.1.1, ip-address 10.7.2 — patch/minor, within existing ranges; full suite 1391/1391 green after). Now 0 high, 0 critical, 9 moderate. Web: 0 high, 2 moderate.</t>
-        </is>
-      </c>
-      <c r="I18" s="33" t="n"/>
+          <t>.github/workflows/ci.yml: npm audit --omit=dev --audit-level=high fails the build (backend + web), alongside tests/lint/build on every push and PR; .github/dependabot.yml: weekly grouped updates for backend + web, security-only for the Expo app, monthly for Actions. Audit 2026-09-25: backend 0 critical / 0 high / 2 moderate; web 0 high / 2 moderate. Fixed that day: multer 2.4.0, nodemailer 9.1.1, ip-address 10.7.2, firebase-admin 13→14.5.0 (push client moved to the modular API; tests/m4-push-client.test.js).</t>
+        </is>
+      </c>
+      <c r="I18" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="J18" s="32" t="inlineStr">
         <is>
-          <t>Still to do: add npm audit to CI + Dependabot (no CI pipeline exists in the repo yet). 8 of the 9 backend moderates come through firebase-admin and need a MAJOR upgrade (v14) — owner decision.</t>
+          <t>Remaining 2 backend moderates: uuid&lt;11.1.1 via gaxios 6 inside @google-cloud/storage (a firebase-admin dependency) — no upstream fix yet; the affected uuid v3/v5/v6-with-buffer path is never called by our code. Dependabot will raise it when Google ships the fix. CI verified locally as a dry run (clean copy, no .env, npm ci): lint, audit, 1394 backend + 54 web tests, web build all green. Takes effect once pushed to GitHub. firebase-admin 14 requires Node 22+ (engines bumped; Node 20 is end-of-life).</t>
         </is>
       </c>
     </row>
@@ -3523,7 +3527,7 @@
       </c>
       <c r="H54" s="32" t="inlineStr">
         <is>
-          <t>app/src/utils/logger.js (debug/info compile out of release builds via __DEV__; no token/OTP/password logged); backend logger redacts sensitive paths (src/utils/logger.js)</t>
+          <t>app/src/utils/logger.js (debug/info compile out of release builds via __DEV__; no token/OTP/password logged); backend logger redacts sensitive paths (src/utils/logger.js); app/tests/logger-redaction.test.js (sensitive keys at any depth, JWT/Bearer/long tokens in strings, errors)</t>
         </is>
       </c>
       <c r="I54" s="33" t="inlineStr">
@@ -3627,7 +3631,7 @@
       </c>
       <c r="H56" s="32" t="inlineStr">
         <is>
-          <t>app/app.config.js: iOS NSAllowsArbitraryLoads false, Android usesCleartextTraffic false; app/src/config/env.js refuses a non-https API URL in any release build (http only for a local dev build)</t>
+          <t>app/app.config.js: iOS NSAllowsArbitraryLoads false, Android usesCleartextTraffic false; app/src/config/env.js refuses a non-https API URL in any release build (http only for a local dev build); app/tests/api-base-url.test.js (release build refuses http incl. localhost; dev build only localhost/LAN)</t>
         </is>
       </c>
       <c r="I56" s="33" t="inlineStr">

</xml_diff>